<commit_message>
Full CRUD Assign 1
</commit_message>
<xml_diff>
--- a/Assignment 1 Report - M02544_2023.xlsx
+++ b/Assignment 1 Report - M02544_2023.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,6 +415,9 @@
       <c r="E1" t="str">
         <v>Ressource</v>
       </c>
+      <c r="F1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -432,8 +435,17 @@
       <c r="E2" t="str">
         <v>https://www.ibm.com/docs/en/integration-bus/10.0.0?topic=services-what-is-web-service</v>
       </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
       <c r="C3" t="str">
         <v>Define service-oriented architecture (SOA) and its significance in backend development</v>
       </c>
@@ -448,6 +460,9 @@
 _x000d_
 </v>
       </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4">
@@ -469,8 +484,17 @@
 _x000d_
 https://aws.amazon.com/compare/the-difference-between-soap-rest/?utm_source=chatgpt.com#what-is-the-difference-between-soap-and-rest--e1bfnw</v>
       </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
       <c r="C5" t="str">
         <v>Discuss the pros and cons of each and when they are most applicable</v>
       </c>
@@ -479,6 +503,9 @@
       </c>
       <c r="E5" t="str">
         <v>https://aws.amazon.com/compare/the-difference-between-soap-rest/</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -497,8 +524,17 @@
       <c r="E6" t="str">
         <v>https://developer.mozilla.org/en-US/docs/Learn_web_development/Core/Scripting/Network_requests</v>
       </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
       <c r="C7" t="str">
         <v>Highlight the role of JSON in REST APIs</v>
       </c>
@@ -507,6 +543,9 @@
       </c>
       <c r="E7" t="str">
         <v>https://www.json.org/json-en.html</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -525,8 +564,17 @@
       <c r="E8" t="str">
         <v>https://developer.mozilla.org/en-US/docs/Glossary/SPA</v>
       </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
       <c r="C9" t="str">
         <v>Explain how SPAs work with backend services to provide dynamic user experiences</v>
       </c>
@@ -535,6 +583,9 @@
       </c>
       <c r="E9" t="str">
         <v>https://learn.microsoft.com/en-us/aspnet/core/client-side/spa/intro</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -555,24 +606,54 @@
       <c r="E10" t="str">
         <v>https://workos.com/blog/security-threats-in-spas-and-how-to-defend-against-them</v>
       </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
+      <c r="A11" t="str">
+        <v>6</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Test</v>
+      </c>
       <c r="C11" t="str">
-        <v>Mention practices like HTTPS, CORS, and authentication strategies (e.g., JWT)</v>
+        <v>Test sub</v>
       </c>
       <c r="D11" t="str">
-        <v>HTTPS encrypts communication between clients and servers, protecting sensitive data from interception. CORS (Cross-Origin Resource Sharing) controls which domains can access backend resources, helping prevent unauthorized cross-origin requests. Authentication strategies such as JWT (JSON Web Tokens) allow secure user authentication and stateless session management. Best practices also include OAuth 2.0, secure cookie handling, token expiration, input validation, rate limiting, and multi-factor authentication (MFA).</v>
+        <v>Test answer</v>
       </c>
       <c r="E11" t="str">
-        <v>https://developer.mozilla.org/en-US/docs/Web/HTTP/CORS</v>
+        <v>http://example.com</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>7</v>
+      </c>
+      <c r="B12" t="str">
+        <v>New Content</v>
+      </c>
+      <c r="C12" t="str">
+        <v>New SubTitle</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Here is a new content</v>
+      </c>
+      <c r="E12" t="str">
+        <v>http://google.com</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="8">
     <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B11"/>
     <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A11"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B4:B5"/>
@@ -580,20 +661,8 @@
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A6:A7"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="E3" r:id="rId2" location="what-is"/>
-    <hyperlink ref="E4" r:id="rId3"/>
-    <hyperlink ref="E5" r:id="rId4"/>
-    <hyperlink ref="E6" r:id="rId5"/>
-    <hyperlink ref="E7" r:id="rId6"/>
-    <hyperlink ref="E8" r:id="rId7"/>
-    <hyperlink ref="E9" r:id="rId8"/>
-    <hyperlink ref="E11" r:id="rId9"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>